<commit_message>
Improve Aruba scraping and brand normalization
</commit_message>
<xml_diff>
--- a/streamlit_data/regional_insights.xlsx
+++ b/streamlit_data/regional_insights.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E152"/>
+  <dimension ref="A1:E153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="C2" t="n">
         <v>3</v>
@@ -465,7 +465,7 @@
         <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>16.91311029719778</v>
+        <v>16.92954930121386</v>
       </c>
     </row>
     <row r="3">
@@ -1269,7 +1269,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Doritos</t>
+          <t>El Charrito</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1281,14 +1281,12 @@
       <c r="D45" t="n">
         <v>1</v>
       </c>
-      <c r="E45" t="n">
-        <v>21.83213295019938</v>
-      </c>
+      <c r="E45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Keebler</t>
+          <t>Doritos</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1298,16 +1296,16 @@
         <v>1</v>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>16.53</v>
+        <v>21.83213295019938</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>El Charrito</t>
+          <t>Keebler</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -1317,9 +1315,11 @@
         <v>1</v>
       </c>
       <c r="D47" t="n">
-        <v>1</v>
-      </c>
-      <c r="E47" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E47" t="n">
+        <v>16.53</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1343,81 +1343,81 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>La Real</t>
+          <t>Pillsbury</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>9</v>
       </c>
       <c r="C49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E49" t="n">
-        <v>12.46</v>
+        <v>7.764285714285714</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Pillsbury</t>
+          <t>La Real</t>
         </is>
       </c>
       <c r="B50" t="n">
         <v>9</v>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>7.764285714285714</v>
+        <v>12.46</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Biskitop</t>
+          <t>Siete</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>8</v>
       </c>
       <c r="C51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D51" t="n">
         <v>2</v>
       </c>
-      <c r="E51" t="inlineStr"/>
+      <c r="E51" t="n">
+        <v>44.83675833138952</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Siete</t>
+          <t>Biskitop</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>8</v>
       </c>
       <c r="C52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
         <v>2</v>
       </c>
-      <c r="E52" t="n">
-        <v>44.83675833138952</v>
-      </c>
+      <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Festival</t>
+          <t>Golden</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -1427,16 +1427,14 @@
         <v>1</v>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
-      </c>
-      <c r="E53" t="n">
-        <v>9.385016025641024</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Golden</t>
+          <t>Nature'S Own</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -1446,14 +1444,16 @@
         <v>1</v>
       </c>
       <c r="D54" t="n">
-        <v>2</v>
-      </c>
-      <c r="E54" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E54" t="n">
+        <v>7.755714285714285</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Walkers</t>
+          <t>Princesa</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -1463,16 +1463,16 @@
         <v>1</v>
       </c>
       <c r="D55" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>97.43589743589745</v>
+        <v>3.535714285714286</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Princesa</t>
+          <t>Biscotto</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -1482,16 +1482,16 @@
         <v>1</v>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>3.535714285714286</v>
+        <v>25</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Kidsmania</t>
+          <t>Walkers</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -1501,14 +1501,16 @@
         <v>1</v>
       </c>
       <c r="D57" t="n">
-        <v>1</v>
-      </c>
-      <c r="E57" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E57" t="n">
+        <v>97.43589743589745</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Nature'S Own</t>
+          <t>Festival</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1521,13 +1523,13 @@
         <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>7.755714285714285</v>
+        <v>9.385016025641024</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Biscotto</t>
+          <t>Kidsmania</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1537,16 +1539,14 @@
         <v>1</v>
       </c>
       <c r="D59" t="n">
-        <v>2</v>
-      </c>
-      <c r="E59" t="n">
-        <v>25</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Sunshine</t>
+          <t>Laurieri</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1556,16 +1556,16 @@
         <v>1</v>
       </c>
       <c r="D60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E60" t="n">
-        <v>9.488333333333333</v>
+        <v>20.65978352354142</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Kugi</t>
+          <t>Mr Bakewell</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1582,24 +1582,26 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Mr Bakewell</t>
+          <t>Cheetos</t>
         </is>
       </c>
       <c r="B62" t="n">
         <v>6</v>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D62" t="n">
         <v>1</v>
       </c>
-      <c r="E62" t="inlineStr"/>
+      <c r="E62" t="n">
+        <v>24.41444882993455</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Laurieri</t>
+          <t>Cadbury</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1611,27 +1613,25 @@
       <c r="D63" t="n">
         <v>2</v>
       </c>
-      <c r="E63" t="n">
-        <v>20.65978352354142</v>
-      </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cheetos</t>
+          <t>Sunshine</t>
         </is>
       </c>
       <c r="B64" t="n">
         <v>6</v>
       </c>
       <c r="C64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>24.41444882993455</v>
+        <v>9.488333333333333</v>
       </c>
     </row>
     <row r="65">
@@ -1654,7 +1654,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Cadbury</t>
+          <t>Kugi</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -1664,14 +1664,14 @@
         <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>La Libanesa</t>
+          <t>Hosttes</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1683,7 +1683,9 @@
       <c r="D67" t="n">
         <v>1</v>
       </c>
-      <c r="E67" t="inlineStr"/>
+      <c r="E67" t="n">
+        <v>36.83418646645511</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1707,20 +1709,20 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Bolletje</t>
+          <t>Schar</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>5</v>
       </c>
       <c r="C69" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D69" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E69" t="n">
-        <v>29.40549939726599</v>
+        <v>24.18904950998269</v>
       </c>
     </row>
     <row r="70">
@@ -1743,26 +1745,26 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Schar</t>
+          <t>Bolletje</t>
         </is>
       </c>
       <c r="B71" t="n">
         <v>5</v>
       </c>
       <c r="C71" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" t="n">
         <v>2</v>
       </c>
-      <c r="D71" t="n">
-        <v>3</v>
-      </c>
       <c r="E71" t="n">
-        <v>24.18904950998269</v>
+        <v>29.40549939726599</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Tiffany</t>
+          <t>Triskits</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1779,7 +1781,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Hosttes</t>
+          <t>La Libanesa</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -1791,14 +1793,12 @@
       <c r="D73" t="n">
         <v>1</v>
       </c>
-      <c r="E73" t="n">
-        <v>36.83418646645511</v>
-      </c>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Triskits</t>
+          <t>Tiffany</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -1834,7 +1834,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Keeber</t>
+          <t>Otis Spunkmeyer</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1844,35 +1844,33 @@
         <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>3</v>
-      </c>
-      <c r="E76" t="n">
-        <v>28.61772083892403</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Takis</t>
+          <t>Nestle</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E77" t="n">
-        <v>41.86</v>
+        <v>41.70528266913809</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Nestle</t>
+          <t>Ovaltine</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1882,16 +1880,16 @@
         <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>41.70528266913809</v>
+        <v>19.9445103354795</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Otis Spunkmeyer</t>
+          <t>Herrs</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1901,14 +1899,16 @@
         <v>1</v>
       </c>
       <c r="D79" t="n">
-        <v>2</v>
-      </c>
-      <c r="E79" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E79" t="n">
+        <v>37.30902864926393</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Ovaltine</t>
+          <t>Buenhorno</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1920,52 +1920,50 @@
       <c r="D80" t="n">
         <v>1</v>
       </c>
-      <c r="E80" t="n">
-        <v>19.9445103354795</v>
-      </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Snyder’S</t>
+          <t>Glutino</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>4</v>
       </c>
       <c r="C81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D81" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E81" t="n">
-        <v>21.8340355175269</v>
+        <v>19.41435404641845</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Glutino</t>
+          <t>Keeber</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>4</v>
       </c>
       <c r="C82" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D82" t="n">
         <v>3</v>
       </c>
       <c r="E82" t="n">
-        <v>19.41435404641845</v>
+        <v>28.61772083892403</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Buenhorno</t>
+          <t>Snyder’S</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1977,31 +1975,33 @@
       <c r="D83" t="n">
         <v>1</v>
       </c>
-      <c r="E83" t="inlineStr"/>
+      <c r="E83" t="n">
+        <v>21.8340355175269</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Herrs</t>
+          <t>Takis</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>4</v>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E84" t="n">
-        <v>37.30902864926393</v>
+        <v>41.86</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Flourish</t>
+          <t>Dux</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -2018,24 +2018,26 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Dux</t>
+          <t>Hostess</t>
         </is>
       </c>
       <c r="B86" t="n">
         <v>3</v>
       </c>
       <c r="C86" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" t="n">
-        <v>1</v>
-      </c>
-      <c r="E86" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="E86" t="n">
+        <v>18.15097496514973</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Waitrose</t>
+          <t>Snyders</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -2045,14 +2047,14 @@
         <v>1</v>
       </c>
       <c r="D87" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Chetos</t>
+          <t>Del-E</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -2062,7 +2064,7 @@
         <v>1</v>
       </c>
       <c r="D88" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E88" t="inlineStr"/>
     </row>
@@ -2088,7 +2090,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Van Der Meulen</t>
+          <t>Flourish</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -2100,14 +2102,12 @@
       <c r="D90" t="n">
         <v>1</v>
       </c>
-      <c r="E90" t="n">
-        <v>12.12155070255629</v>
-      </c>
+      <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Snyders</t>
+          <t>Waitrose</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -2117,33 +2117,33 @@
         <v>1</v>
       </c>
       <c r="D91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Hostess</t>
+          <t>Van Der Meulen</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D92" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E92" t="n">
-        <v>18.15097496514973</v>
+        <v>12.12155070255629</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Del-E</t>
+          <t>Chetos</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -2153,14 +2153,14 @@
         <v>1</v>
       </c>
       <c r="D93" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Voortman</t>
+          <t>Ricola</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -2173,13 +2173,13 @@
         <v>1</v>
       </c>
       <c r="E94" t="n">
-        <v>20.17345399698341</v>
+        <v>7.351955307262569</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Ricola</t>
+          <t>Wala</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -2191,14 +2191,12 @@
       <c r="D95" t="n">
         <v>1</v>
       </c>
-      <c r="E95" t="n">
-        <v>7.351955307262569</v>
-      </c>
+      <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Vigo</t>
+          <t>Voortman</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -2211,13 +2209,13 @@
         <v>1</v>
       </c>
       <c r="E96" t="n">
-        <v>9.433248720978664</v>
+        <v>20.17345399698341</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Wala</t>
+          <t>Werther’S</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -2234,7 +2232,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Werther’S</t>
+          <t>Vigo</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -2246,12 +2244,14 @@
       <c r="D98" t="n">
         <v>1</v>
       </c>
-      <c r="E98" t="inlineStr"/>
+      <c r="E98" t="n">
+        <v>9.433248720978664</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Willie</t>
+          <t>Sara Lee</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -2263,12 +2263,14 @@
       <c r="D99" t="n">
         <v>1</v>
       </c>
-      <c r="E99" t="inlineStr"/>
+      <c r="E99" t="n">
+        <v>24.085</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Beivita</t>
+          <t>Dried</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -2278,16 +2280,14 @@
         <v>1</v>
       </c>
       <c r="D100" t="n">
-        <v>1</v>
-      </c>
-      <c r="E100" t="n">
-        <v>35.19230769230769</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Tuc</t>
+          <t>Willie</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -2299,14 +2299,12 @@
       <c r="D101" t="n">
         <v>1</v>
       </c>
-      <c r="E101" t="n">
-        <v>7.575418994413408</v>
-      </c>
+      <c r="E101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Soldanza</t>
+          <t>Beivita</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -2318,12 +2316,14 @@
       <c r="D102" t="n">
         <v>1</v>
       </c>
-      <c r="E102" t="inlineStr"/>
+      <c r="E102" t="n">
+        <v>35.19230769230769</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Cheez</t>
+          <t>Tuc</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -2335,12 +2335,14 @@
       <c r="D103" t="n">
         <v>1</v>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="n">
+        <v>7.575418994413408</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Sara Lee</t>
+          <t>Soldanza</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -2352,14 +2354,12 @@
       <c r="D104" t="n">
         <v>1</v>
       </c>
-      <c r="E104" t="n">
-        <v>24.085</v>
-      </c>
+      <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Knotts</t>
+          <t>Glad</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -2376,7 +2376,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Danisha</t>
+          <t>Cheez</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -2393,7 +2393,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Hills</t>
+          <t>Mars</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -2410,7 +2410,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Dairy</t>
+          <t>Danisha</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -2427,7 +2427,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>La Tortilla Factory</t>
+          <t>Hinged</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -2440,13 +2440,13 @@
         <v>1</v>
       </c>
       <c r="E109" t="n">
-        <v>21.71</v>
+        <v>1.907848055928269</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Hinged</t>
+          <t>Hills</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -2458,14 +2458,12 @@
       <c r="D110" t="n">
         <v>1</v>
       </c>
-      <c r="E110" t="n">
-        <v>1.907848055928269</v>
-      </c>
+      <c r="E110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Crunchmaster</t>
+          <t>La Tortilla Factory</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -2478,7 +2476,7 @@
         <v>1</v>
       </c>
       <c r="E111" t="n">
-        <v>51.37009840929231</v>
+        <v>21.71</v>
       </c>
     </row>
     <row r="112">
@@ -2503,14 +2501,14 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Mars</t>
+          <t>Nature Valley</t>
         </is>
       </c>
       <c r="B113" t="n">
         <v>2</v>
       </c>
       <c r="C113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D113" t="n">
         <v>1</v>
@@ -2520,14 +2518,14 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Nature Valley</t>
+          <t>Dairy</t>
         </is>
       </c>
       <c r="B114" t="n">
         <v>2</v>
       </c>
       <c r="C114" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D114" t="n">
         <v>1</v>
@@ -2537,7 +2535,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Dried</t>
+          <t>Crunchmaster</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -2547,14 +2545,16 @@
         <v>1</v>
       </c>
       <c r="D115" t="n">
-        <v>2</v>
-      </c>
-      <c r="E115" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E115" t="n">
+        <v>51.37009840929231</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Glad</t>
+          <t>Knotts</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -2588,7 +2588,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Vegefarm</t>
+          <t>Badia</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -2600,14 +2600,12 @@
       <c r="D118" t="n">
         <v>1</v>
       </c>
-      <c r="E118" t="n">
-        <v>27.42714334124026</v>
-      </c>
+      <c r="E118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Kimberley's Bakeshoppe</t>
+          <t>King's Hawaiian</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -2624,7 +2622,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Highland</t>
+          <t>Holiday</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -2641,7 +2639,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Hershey</t>
+          <t>Kimberley's Bakeshoppe</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -2653,14 +2651,12 @@
       <c r="D121" t="n">
         <v>1</v>
       </c>
-      <c r="E121" t="n">
-        <v>19.07848055928269</v>
-      </c>
+      <c r="E121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Goldfish</t>
+          <t>Twizzlers</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -2672,14 +2668,12 @@
       <c r="D122" t="n">
         <v>1</v>
       </c>
-      <c r="E122" t="n">
-        <v>15.39664804469274</v>
-      </c>
+      <c r="E122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Haagen Daz</t>
+          <t>Hollandia</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -2691,12 +2685,14 @@
       <c r="D123" t="n">
         <v>1</v>
       </c>
-      <c r="E123" t="inlineStr"/>
+      <c r="E123" t="n">
+        <v>52.34878150009826</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Twizzlers</t>
+          <t>Jumbo</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -2708,12 +2704,14 @@
       <c r="D124" t="n">
         <v>1</v>
       </c>
-      <c r="E124" t="inlineStr"/>
+      <c r="E124" t="n">
+        <v>11.48504273504274</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Haribo</t>
+          <t>Cusano´s</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -2730,7 +2728,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Holiday</t>
+          <t>Triscuit</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -2742,12 +2740,14 @@
       <c r="D126" t="n">
         <v>1</v>
       </c>
-      <c r="E126" t="inlineStr"/>
+      <c r="E126" t="n">
+        <v>21.76632743949854</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Give &amp; Go</t>
+          <t>Ducales</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -2759,12 +2759,14 @@
       <c r="D127" t="n">
         <v>1</v>
       </c>
-      <c r="E127" t="inlineStr"/>
+      <c r="E127" t="n">
+        <v>21.76632743949854</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Ducales</t>
+          <t>Give &amp; Go</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -2776,14 +2778,12 @@
       <c r="D128" t="n">
         <v>1</v>
       </c>
-      <c r="E128" t="n">
-        <v>21.76632743949854</v>
-      </c>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Triscuit</t>
+          <t>Lewis Bake Shop</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -2796,13 +2796,13 @@
         <v>1</v>
       </c>
       <c r="E129" t="n">
-        <v>21.76632743949854</v>
+        <v>3.284356678113635</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Hollandia</t>
+          <t>Vegefarm</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -2815,13 +2815,13 @@
         <v>1</v>
       </c>
       <c r="E130" t="n">
-        <v>52.34878150009826</v>
+        <v>27.42714334124026</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Jumbo</t>
+          <t>Chester</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -2833,14 +2833,12 @@
       <c r="D131" t="n">
         <v>1</v>
       </c>
-      <c r="E131" t="n">
-        <v>11.48504273504274</v>
-      </c>
+      <c r="E131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Double Duty</t>
+          <t>Marie</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -2857,7 +2855,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Cho Cho</t>
+          <t>Ortega</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -2869,12 +2867,14 @@
       <c r="D133" t="n">
         <v>1</v>
       </c>
-      <c r="E133" t="inlineStr"/>
+      <c r="E133" t="n">
+        <v>10.91045974485786</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>King's Hawaiian</t>
+          <t>Oscar Mayer</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -2886,12 +2886,14 @@
       <c r="D134" t="n">
         <v>1</v>
       </c>
-      <c r="E134" t="inlineStr"/>
+      <c r="E134" t="n">
+        <v>21.70707121411719</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Members Selection</t>
+          <t>Hershey</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -2903,12 +2905,14 @@
       <c r="D135" t="n">
         <v>1</v>
       </c>
-      <c r="E135" t="inlineStr"/>
+      <c r="E135" t="n">
+        <v>19.07848055928269</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Ortega</t>
+          <t>Cho Cho</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -2920,14 +2924,12 @@
       <c r="D136" t="n">
         <v>1</v>
       </c>
-      <c r="E136" t="n">
-        <v>10.91045974485786</v>
-      </c>
+      <c r="E136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Oscar Mayer</t>
+          <t>Nerds</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -2939,14 +2941,12 @@
       <c r="D137" t="n">
         <v>1</v>
       </c>
-      <c r="E137" t="n">
-        <v>21.70707121411719</v>
-      </c>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Nerds</t>
+          <t>Highland</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -2963,7 +2963,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Choppers</t>
+          <t>Haribo</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -2980,7 +2980,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Ferrero</t>
+          <t>Haagen Daz</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -2997,7 +2997,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Chowmein</t>
+          <t>Post</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -3009,12 +3009,14 @@
       <c r="D141" t="n">
         <v>1</v>
       </c>
-      <c r="E141" t="inlineStr"/>
+      <c r="E141" t="n">
+        <v>7.51</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Cloverhill</t>
+          <t>Double Duty</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -3031,7 +3033,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Mcvitie'S</t>
+          <t>Reynolds</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -3043,14 +3045,12 @@
       <c r="D143" t="n">
         <v>1</v>
       </c>
-      <c r="E143" t="n">
-        <v>37.62485187066193</v>
-      </c>
+      <c r="E143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Badia</t>
+          <t>Choppers</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -3067,7 +3067,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Reynolds</t>
+          <t>Ferrero</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -3084,7 +3084,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Marie</t>
+          <t>Ruffles</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -3096,12 +3096,14 @@
       <c r="D146" t="n">
         <v>1</v>
       </c>
-      <c r="E146" t="inlineStr"/>
+      <c r="E146" t="n">
+        <v>20.12215858124287</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Ruffles</t>
+          <t>Chowmein</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -3113,14 +3115,12 @@
       <c r="D147" t="n">
         <v>1</v>
       </c>
-      <c r="E147" t="n">
-        <v>20.12215858124287</v>
-      </c>
+      <c r="E147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Lewis Bake Shop</t>
+          <t>Goldfish</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -3133,13 +3133,13 @@
         <v>1</v>
       </c>
       <c r="E148" t="n">
-        <v>3.284356678113635</v>
+        <v>15.39664804469274</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Cusano´s</t>
+          <t>Cloverhill</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -3175,7 +3175,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Chester</t>
+          <t>Members Selection</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -3192,19 +3192,38 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
+          <t>Mcvitie'S</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+      <c r="E152" t="n">
+        <v>37.62485187066193</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
           <t>Fernandes</t>
         </is>
       </c>
-      <c r="B152" t="n">
-        <v>1</v>
-      </c>
-      <c r="C152" t="n">
-        <v>1</v>
-      </c>
-      <c r="D152" t="n">
-        <v>1</v>
-      </c>
-      <c r="E152" t="inlineStr"/>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="n">
+        <v>1</v>
+      </c>
+      <c r="E153" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>